<commit_message>
v16.4: docs(edim): C13 완료 — RTM 추적 범위 규칙 명문화 (RTM v0.2)
- RTM 문서정보 시트에 추적 범위 명문화: RTM=요구사항(REQ-F/NFR) 중심 추적, 구현 증분(B~G 배치)=EDIM_미구현기능목록.md 가 배치 단위 추적, RTM 형식 확장 없음
- make_rtm_xlsx.py 재생성 — 추적 180행·커버리지 179/179 유지
</commit_message>
<xml_diff>
--- a/edim-ai-blueprint/docs/EDIM_요구사항추적표.xlsx
+++ b/edim-ai-blueprint/docs/EDIM_요구사항추적표.xlsx
@@ -472,7 +472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:C9"/>
+  <dimension ref="B2:C10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="2" max="2"/>
@@ -494,7 +494,7 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>v0.1 (자동 생성)</t>
+          <t>v0.2 (자동 생성)</t>
         </is>
       </c>
     </row>
@@ -506,7 +506,7 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-07 (v0.2 갱신 2026-07-15)</t>
         </is>
       </c>
     </row>
@@ -537,22 +537,34 @@
     <row r="8">
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>추적 행</t>
+          <t>추적 범위</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>180건 (요구사항 50 × 기능 매핑)</t>
+          <t>본 RTM 은 요구사항(REQ-F/NFR) 중심 추적만 담당한다. 요구사항 확정 이후의 구현 증분(B/C/D/E/F/G 배치)은 docs/EDIM_미구현기능목록.md 가 배치 단위(구현·검증·버전)로 추적하며 RTM 형식을 확장하지 않는다 (C13 규칙, 2026-07-15 명문화).</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="B9" s="2" t="inlineStr">
         <is>
+          <t>추적 행</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>180건 (요구사항 50 × 기능 매핑)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="2" t="inlineStr">
+        <is>
           <t>커버리지</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t>기능 179/179 연결 · 미연결 0건 · 해석불가 0건 (커버리지 시트 참조)</t>
         </is>

</xml_diff>